<commit_message>
Excel templates: dropdown lists for the option columns
- Timeline (countries_template.xlsx): Country 1-5 (240 Arabic names with
  short common forms; typing other names, also English, still allowed),
  Intro, Map style, Guess, Mode, Theme, Music (strict) and Unit (suggested)
- Multiple Choice (questions_template.xlsx): Correct (A-D / أ-د)
- Values live on a hidden "Lists" sheet; each dropdown cell shows a tip
- Batch music names now match case-insensitively

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6opBUnfaHre2KUCGjz4Pv
</commit_message>
<xml_diff>
--- a/projects/countries_template.xlsx
+++ b/projects/countries_template.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Videos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to fill" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1195,6 +1196,32 @@
       <c r="U11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="8">
+    <dataValidation sqref="B2:B500 D2:D500 F2:F500 H2:H500 J2:J500" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Pick a country, or type one (Arabic or English)" type="list">
+      <formula1>=Lists!$A$1:$A$240</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="hook = text intro, vs = flags battle" type="list">
+      <formula1>=Lists!$B$1:$B$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="auto picks the best style from the numbers" type="list">
+      <formula1>=Lists!$C$1:$C$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Show the guess moment (3 choices + timer)?" type="list">
+      <formula1>=Lists!$D$1:$D$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Pick a unit or type your own" type="list">
+      <formula1>=Lists!$E$1:$E$11</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = number line" type="list">
+      <formula1>=Lists!$F$1:$F$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = the theme set in the app" type="list">
+      <formula1>=Lists!$G$1:$G$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = the music set in the app" type="list">
+      <formula1>=Lists!$H$1:$H$10</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1205,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1221,70 +1248,2003 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Country 1-5: Arabic or English name (مصر / Egypt) or the 3-letter code (EGY). 2 to 5 countries per row.</t>
+          <t>Click a cell to get its dropdown list: Country (or type any name, also in English), Intro, Map style, Guess,</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Value 1-5: the official area in km² (or any number: heights, prices…). 2,149,690 or ٢١٤٩٦٩٠ are fine.</t>
+          <t xml:space="preserve">   Unit, Mode, Theme and Music.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hook / Reveal: new lines with Alt+Enter (or ' | '). Start a line with [gold], [green], [red]… to colour it.</t>
+          <t>Country 1-5: Arabic or English name (مصر / Egypt) or the 3-letter code (EGY). 2 to 5 countries per row.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Leave Hook / Reveal empty and they are written automatically from the numbers.</t>
+          <t>Value 1-5: the official area in km² (or any number: heights, prices…). 2,149,690 or ٢١٤٩٦٩٠ are fine.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Intro: hook (text) or vs (flags battle).  Map style: auto, overlay, tiles, side.  Guess: yes / no.</t>
+          <t>Hook / Reveal: new lines with Alt+Enter (or ' | '). Start a line with [gold], [green], [red]… to colour it.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   auto = tile fill when one country is 20× bigger or more, side by side within 1.5×, overlay otherwise.</t>
+          <t xml:space="preserve">   Leave Hook / Reveal empty and they are written automatically from the numbers.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ending question: the question for the next video (tease the next row!).</t>
+          <t>Intro: hook (text) or vs (flags battle).  Map style: auto, overlay, tiles, side.  Guess: yes / no.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Optional: Unit (default كم²), Mode (number line / calendar years), Theme (e.g. Ocean), Music.</t>
+          <t xml:space="preserve">   auto = tile fill when one country is 20× bigger or more, side by side within 1.5×, overlay otherwise.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Not a country? Add a 'Name 1' column (and leave Country 1 empty), e.g. برج خليفة with Value 828 and Unit متر.</t>
+          <t>Ending question: the question for the next video (tease the next row!).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Optional: Unit (default كم²), Mode (number line / calendar years), Theme (e.g. Ocean), Music.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Not a country? Add a 'Name 1' column (and leave Country 1 empty), e.g. برج خليفة with Value 828 and Unit متر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Everything else (handle, music, font, ending call-to-action…) comes from the app's 🎨 Style &amp; sound and 🔚 Ending.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H240"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>آيسلندا</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hook</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>كم²</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>number line</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Night Sky</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Tension</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>أذربيجان</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>overlay</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>متر</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>calendar</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Desert Night</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Mystery</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>أراض فرنسية جنوبية وأنتارتيكية</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>tiles</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>كم</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>years ago</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Emerald</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Calm</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>أرمينيا</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>side</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>م²</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Deep Purple</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pulse</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>أروبا</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>كغ</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Charcoal</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Quiz Show</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>أستراليا</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Royal Blue</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Bright Pop</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>أفغانستان</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>km²</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ocean</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lo-fi Chill</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>أقاليم المحيط الهندي الأسترالية</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Midnight Gold</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ألبانيا</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>km</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Crimson</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ألمانيا</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Slate</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>أمريكا</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>أنتيغوا وباربودا</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Rose Wine</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>أندورا</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Cyber Night</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>أنغولا</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>أنغويلا</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>أوزبكستان</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>أوغندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>أوكرانيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>إثيوبيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>إريتريا</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>إسبانيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>إستونيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>إسرائيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>إسواتيني</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>إقليم المحيط الهندي البريطاني</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>إندونيسيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>إيران</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>إيطاليا</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>الأرجنتين</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>الأردن</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>الأوروغواي</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>الإكوادور</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>الإمارات</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>البحرين</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>البرازيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>البرتغال</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>البوسنة والهرسك</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>التشيك</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>الجبل الأسود</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>الجزائر</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>الدنمارك</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>الرأس الأخضر</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>السعودية</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>السلفادور</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>السنغال</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>السودان</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>السويد</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>الصحراء الغربية</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>الصومال</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>الصين</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>العراق</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>الغابون</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>الفاتيكان</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>الفلبين</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>القارة القطبية الجنوبية</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>الكاميرون</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>الكويت</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>المالديف</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>المجر</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>المغرب</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>المكسيك</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>النرويج</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>النمسا</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>النيجر</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>الهند</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>اليابان</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>اليمن</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>اليونان</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>بابوا غينيا الجديدة</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>باراغواي</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>باربادوس</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>باكستان</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>بالاو</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>باهاماس</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>برمودا</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>بروناي</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>بريطانيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>بلجيكا</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>بلغاريا</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>بليز</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>بنغلاديش</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>بنما</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>بنين</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>بوتان</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>بوتسوانا</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>بورتوريكو</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>بوركينا فاسو</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>بوروندي</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>بولندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>بوليفيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>بولينزيا الفرنسية</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>بيرو</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>بيلاروسيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>تايلاند</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>تايوان</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>تجمع سان مارتين</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>تركمانستان</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>تركيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ترينيداد وتوباغو</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>تشاد</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>تشيلي</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>تنزانيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>توغو</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>توفالو</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>تونس</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>تونغا</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>تيمور الشرقية</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>جامايكا</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>جزر أولاند</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>جزر العذراء الأمريكية</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>جزر العذراء البريطانية</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>جزر القمر</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>جزر بيتكيرن</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>جزر توركس وكايكوس</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>جزر سليمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>جزر فارو</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>جزر فوكلاند</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>جزر كايمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>جزر كوك</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>جزر مارشال</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>جزر ماريانا الشمالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>جزيرة مان</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>جزيرة نورفولك</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>جزيرة هيرد وجزر ماكدونالد</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>جمهورية أفريقيا الوسطى</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>جمهورية أيرلندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>جمهورية الدومينيكان</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>جمهورية الكونغو</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>جمهورية الكونغو الديمقراطية</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>جنوب أفريقيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>جنوب السودان</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>جورجيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>جورجيا الجنوبية وجزر ساندويتش الجنوبية</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>جيبوتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>جيرزي</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>دومينيكا</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>رواندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>روسيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>رومانيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>زامبيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>زيمبابوي</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>ساحل العاج</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>ساموا</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>ساموا الأمريكية</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>سان بارتيلمي</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>سان بيير وميكلون</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>سان مارينو</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>سانت فينسنت والغرينادين</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>سانت كيتس ونيفيس</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>سانت لوسيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>سانت هيلينا</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>ساو تومي وبرينسيب</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>سريلانكا</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>سلوفاكيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>سلوفينيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>سنغافورة</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>سوريا</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>سورينام</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>سويسرا</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>سيراليون</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>سيشل</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>سينت مارتن</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>صربيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>صوماليلاند</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>طاجيكستان</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>عمان</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>غامبيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>غانا</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>غرينادا</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>غرينلاند</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>غواتيمالا</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>غوام</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>غيانا</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>غيرنزي</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>غينيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>غينيا الاستوائية</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>غينيا بيساو</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>فانواتو</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>فرنسا</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>فلسطين</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>فنزويلا</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>فنلندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>فيتنام</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>فيجي</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>قبرص</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>قبرص الشمالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>قطر</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>قيرغيزستان</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>كازاخستان</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>كاليدونيا الجديدة</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>كرواتيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>كمبوديا</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>كندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>كوبا</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>كوراساو</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>كوريا الجنوبية</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>كوريا الشمالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>كوستاريكا</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>كوسوفو</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>كولومبيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>كيريباتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>كينيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>لاتفيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>لاوس</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>لبنان</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>لوكسمبورغ</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>ليبيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>ليبيريا</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>ليتوانيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>ليختنشتاين</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>ليسوتو</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>ماكاو</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>مالاوي</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>مالطا</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>مالي</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>ماليزيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>مدغشقر</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>مصر</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>مقدونيا الشمالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>منغوليا</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>موريتانيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>موريشيوس</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>موزمبيق</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>مولدوفا</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>موناكو</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>مونتسرات</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>ميانمار</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>ناميبيا</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>ناورو</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>نيبال</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>نيجيريا</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>نيكاراغوا</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>نيوزيلندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>نييوي</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>هايتي</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>هندوراس</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>هولندا</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>هونغ كونغ</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>واليس وفوتونا</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>ولايات ميكرونيسيا المتحدة</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Countries template: left-to-right sheet, Doubt / Doubt subtitle / Compare title columns
- The sheet runs left to right; Arabic text cells stay right-aligned with
  right-to-left reading order
- New columns after Hook: Doubt (the big word, e.g. مستحيل؟), Doubt subtitle
  and Compare title, pre-filled in the 10 example rows; empty = app text
- Template columns are now laid out by header name

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U6opBUnfaHre2KUCGjz4Pv
</commit_message>
<xml_diff>
--- a/projects/countries_template.xlsx
+++ b/projects/countries_template.xlsx
@@ -59,16 +59,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:X11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -450,15 +453,18 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,45 +530,60 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Doubt</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Doubt subtitle</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Compare title</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Reveal</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Intro</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Map style</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Guess</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Ending question</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Mode</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Theme</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Music</t>
         </is>
@@ -611,35 +632,50 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
+          <t>مستحيل؟</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
           <t>[red]لبنان يدخل في السعودية
 206 مرات!</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>أيهما أكبر:
 [gold]غرينلاند أم السعودية؟</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="inlineStr"/>
-      <c r="U2" s="2" t="inlineStr"/>
+      <c r="U2" s="4" t="inlineStr"/>
+      <c r="V2" s="4" t="inlineStr"/>
+      <c r="W2" s="4" t="inlineStr"/>
+      <c r="X2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -678,35 +714,50 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
+          <t>هل تصدق؟</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
           <t>[gold]الفرق بينهما
 أقل من 1%!</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="S3" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>مصر أقرب في المساحة
 [gold]إلى من؟</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr"/>
-      <c r="U3" s="2" t="inlineStr"/>
+      <c r="U3" s="4" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr"/>
+      <c r="W3" s="4" t="inlineStr"/>
+      <c r="X3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -751,35 +802,50 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
+          <t>مستحيل؟</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
           <t>[green]السعودية أكبر من
 ضعف مساحة مصر!</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>كم بحرين تدخل
 [gold]في الكويت؟</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="inlineStr"/>
-      <c r="U4" s="2" t="inlineStr"/>
+      <c r="U4" s="4" t="inlineStr"/>
+      <c r="V4" s="4" t="inlineStr"/>
+      <c r="W4" s="4" t="inlineStr"/>
+      <c r="X4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -810,32 +876,47 @@
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>حقًا؟</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="S5" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>الأردن أم البرتغال:
 [gold]أيهما أكبر؟</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="inlineStr"/>
+      <c r="U5" s="4" t="inlineStr"/>
+      <c r="V5" s="4" t="inlineStr"/>
+      <c r="W5" s="4" t="inlineStr"/>
+      <c r="X5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -866,32 +947,47 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>مستحيل؟</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>غانا أم بريطانيا:
 [gold]أيهما أكبر؟</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr"/>
-      <c r="U6" s="2" t="inlineStr"/>
+      <c r="U6" s="4" t="inlineStr"/>
+      <c r="V6" s="4" t="inlineStr"/>
+      <c r="W6" s="4" t="inlineStr"/>
+      <c r="X6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -922,32 +1018,47 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>هل تصدق؟</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="S7" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>أكبر 3 دول عربية:
 [gold]من الأولى؟</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr"/>
-      <c r="U7" s="2" t="inlineStr"/>
+      <c r="U7" s="4" t="inlineStr"/>
+      <c r="V7" s="4" t="inlineStr"/>
+      <c r="W7" s="4" t="inlineStr"/>
+      <c r="X7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -991,35 +1102,50 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t>مستحيل؟</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
           <t>[gold]الجزائر الأولى
 بفارق صغير!</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="R8" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>كم كويت تدخل
 [gold]في العراق؟</t>
         </is>
       </c>
-      <c r="R8" s="2" t="inlineStr"/>
-      <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="inlineStr"/>
-      <c r="U8" s="2" t="inlineStr"/>
+      <c r="U8" s="4" t="inlineStr"/>
+      <c r="V8" s="4" t="inlineStr"/>
+      <c r="W8" s="4" t="inlineStr"/>
+      <c r="X8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1050,32 +1176,47 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>حقًا؟</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="S9" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q9" s="2" t="inlineStr">
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t>كم تونس تدخل
 [gold]في ليبيا؟</t>
         </is>
       </c>
-      <c r="R9" s="2" t="inlineStr"/>
-      <c r="S9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="inlineStr"/>
-      <c r="U9" s="2" t="inlineStr"/>
+      <c r="U9" s="4" t="inlineStr"/>
+      <c r="V9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="inlineStr"/>
+      <c r="X9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1106,32 +1247,47 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>مستحيل؟</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="S10" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q10" s="2" t="inlineStr">
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>الإمارات وعُمان واليمن:
 [gold]رتّبها حسب المساحة!</t>
         </is>
       </c>
-      <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr"/>
+      <c r="U10" s="4" t="inlineStr"/>
+      <c r="V10" s="4" t="inlineStr"/>
+      <c r="W10" s="4" t="inlineStr"/>
+      <c r="X10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1168,57 +1324,72 @@
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>هل تصدق؟</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
+          <t>تابع المساحة…</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>بالحجم الحقيقي…</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="R11" s="4" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="S11" s="4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="Q11" s="2" t="inlineStr">
+      <c r="T11" s="2" t="inlineStr">
         <is>
           <t>اكتب دولتين
 [gold]لنقارنهما!</t>
         </is>
       </c>
-      <c r="R11" s="2" t="inlineStr"/>
-      <c r="S11" s="2" t="inlineStr"/>
-      <c r="T11" s="2" t="inlineStr"/>
-      <c r="U11" s="2" t="inlineStr"/>
+      <c r="U11" s="4" t="inlineStr"/>
+      <c r="V11" s="4" t="inlineStr"/>
+      <c r="W11" s="4" t="inlineStr"/>
+      <c r="X11" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="8">
     <dataValidation sqref="B2:B500 D2:D500 F2:F500 H2:H500 J2:J500" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Pick a country, or type one (Arabic or English)" type="list">
       <formula1>=Lists!$A$1:$A$240</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="hook = text intro, vs = flags battle" type="list">
+    <dataValidation sqref="Q2:Q500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="hook = text intro, vs = flags battle" type="list">
       <formula1>=Lists!$B$1:$B$2</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="auto picks the best style from the numbers" type="list">
+    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="auto picks the best style from the numbers" type="list">
       <formula1>=Lists!$C$1:$C$4</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Show the guess moment (3 choices + timer)?" type="list">
+    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Show the guess moment (3 choices + timer)?" type="list">
       <formula1>=Lists!$D$1:$D$2</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Pick a unit or type your own" type="list">
+    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Pick a unit or type your own" type="list">
       <formula1>=Lists!$E$1:$E$11</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = number line" type="list">
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = number line" type="list">
       <formula1>=Lists!$F$1:$F$3</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = the theme set in the app" type="list">
+    <dataValidation sqref="W2:W500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = the theme set in the app" type="list">
       <formula1>=Lists!$G$1:$G$13</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = the music set in the app" type="list">
+    <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not in the list" error="Pick one of the choices from the dropdown list." prompt="Empty = the music set in the app" type="list">
       <formula1>=Lists!$H$1:$H$10</formula1>
     </dataValidation>
   </dataValidations>
@@ -1232,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1283,47 +1454,61 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Leave Hook / Reveal empty and they are written automatically from the numbers.</t>
+          <t>Doubt: the big word after the hook (مستحيل؟ / هل تصدق؟ / حقًا؟), Doubt subtitle: the small line under it.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Intro: hook (text) or vs (flags battle).  Map style: auto, overlay, tiles, side.  Guess: yes / no.</t>
+          <t>Compare title: the title over the maps / bars (بالحجم الحقيقي…). Empty = the app's text.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   auto = tile fill when one country is 20× bigger or more, side by side within 1.5×, overlay otherwise.</t>
+          <t xml:space="preserve">   Leave Hook / Reveal empty and they are written automatically from the numbers.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ending question: the question for the next video (tease the next row!).</t>
+          <t>Intro: hook (text) or vs (flags battle).  Map style: auto, overlay, tiles, side.  Guess: yes / no.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Optional: Unit (default كم²), Mode (number line / calendar years), Theme (e.g. Ocean), Music.</t>
+          <t xml:space="preserve">   auto = tile fill when one country is 20× bigger or more, side by side within 1.5×, overlay otherwise.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Not a country? Add a 'Name 1' column (and leave Country 1 empty), e.g. برج خليفة with Value 828 and Unit متر.</t>
+          <t>Ending question: the question for the next video (tease the next row!).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>Optional: Unit (default كم²), Mode (number line / calendar years), Theme (e.g. Ocean), Music.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Not a country? Add a 'Name 1' column (and leave Country 1 empty), e.g. برج خليفة with Value 828 and Unit متر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Everything else (handle, music, font, ending call-to-action…) comes from the app's 🎨 Style &amp; sound and 🔚 Ending.</t>
         </is>

</xml_diff>